<commit_message>
test(t2): golden 比对脚本 + 真实 2025-12 基线 + 问题行告警
</commit_message>
<xml_diff>
--- a/tests/golden/invoice_income_exporter/2026年度开票收入.xlsx
+++ b/tests/golden/invoice_income_exporter/2026年度开票收入.xlsx
@@ -21,6 +21,10 @@
     <sheet name="202601" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="未收款明细2026年12月" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="未收款明细2025年12月" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="未收款明细2024年12月" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="未收款明细2023年12月" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="未收款明细2022年12月" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="未收款明细2020年12月" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -80,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -94,6 +98,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1081,6 +1094,1249 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:E59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>浙江震天律师事务所</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2025年度开具发票截止2025年12月律师未收款明细表</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>姓名</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>发票开具月份</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>对方抬头</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>未收款金额</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>章山山</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>1月</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市越城区体育中心</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>107000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>应佳奇</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>2月</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>罗苗君（个人）</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>周利生</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>3月</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>安徽钛韧建筑工程有限公司</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>徐志庆</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>4月</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市商旅文化发展有限公司</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>116000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>柳立中</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>4月</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市商旅文化发展有限公司</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>22900</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>宣浙军</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>4月</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>俞智燚（个人）</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>19000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>陈娟</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>4月</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>郑建新（个人）</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>27900</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>117900</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>周士杰</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>中国农业银行股份有限公司绍兴分行</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>37000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n"/>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>中国农业银行股份有限公司绍兴分行</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n"/>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>中国农业银行股份有限公司绍兴分行</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n"/>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>中国农业银行股份有限公司绍兴分行</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n"/>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>中国农业银行股份有限公司绍兴分行</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>中国农业银行股份有限公司绍兴分行</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n"/>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>中国农业银行股份有限公司绍兴分行</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n"/>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>中国农业银行股份有限公司绍兴分行</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n"/>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>中国农业银行股份有限公司绍兴分行</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n"/>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>中国农业银行股份有限公司绍兴分行</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n"/>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>中国农业银行股份有限公司绍兴分行</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>中国农业银行股份有限公司绍兴分行</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>陈娟</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>6月</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>沈佳栋（个人）</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>90000</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>117900</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>徐志庆</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>6月</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市通华电器有限公司</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>29000</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>116000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n"/>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>6月</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市未来公用事业产业发展有限公司</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>傅强</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>6月</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市未来公用事业产业发展有限公司</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>28000</v>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>166000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>丁祥锋</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>6月</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>崔张华（个人）</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>章山山</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>7月</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>中国工商银行股份有限公司绍兴分行</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>107000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>宣浙军</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>7月</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>俞智燚（个人）</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>19000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>朱云</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>8月</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市越城区东湖街道杨浜村村民委员会</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>25522.4</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>105522.4</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>柳立中</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>9月</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市清能环保有限公司</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>22900</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n"/>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>9月</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市清能环保有限公司</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="n">
+        <v>5900</v>
+      </c>
+      <c r="E32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>傅锦琪</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>9月</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市清能环保有限公司</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>19000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>柳立中</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>9月</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市清能环保有限公司</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E34" s="9" t="n">
+        <v>22900</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>徐志庆</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>9月</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市清能环保有限公司</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E35" s="9" t="n">
+        <v>116000</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>柳立中</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>9月</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市清能环保有限公司</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="n">
+        <v>5500</v>
+      </c>
+      <c r="E36" s="9" t="n">
+        <v>22900</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n"/>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>9月</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市清能环保有限公司</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>章山山</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>10月</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市越城区体育中心</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E38" s="9" t="n">
+        <v>107000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>王建</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>10月</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>魏晓琴等（个人）</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="n">
+        <v>23000</v>
+      </c>
+      <c r="E39" s="9" t="n">
+        <v>33000</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>徐志庆</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>10月</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>绍兴柯桥兆山水泥有限公司</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E40" s="9" t="n">
+        <v>116000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>章山山</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市越城区体育中心</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E41" s="9" t="n">
+        <v>107000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n"/>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>绍兴文理学院后勤发展有限公司</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>王建</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>金超权（个人）</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E43" s="9" t="n">
+        <v>33000</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>周士杰</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市商旅文化发展有限公司</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="n">
+        <v>19000</v>
+      </c>
+      <c r="E44" s="9" t="n">
+        <v>37000</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>傅锦琪</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市商旅文化发展有限公司</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="n">
+        <v>16000</v>
+      </c>
+      <c r="E45" s="9" t="n">
+        <v>19000</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>朱琰芳</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>绍兴袍江基础设施运营有限公司</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="n">
+        <v>5400</v>
+      </c>
+      <c r="E46" s="9" t="n">
+        <v>5400</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>余佳艳</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>绍兴袍江基础设施运营有限公司</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="n">
+        <v>12600</v>
+      </c>
+      <c r="E47" s="9" t="n">
+        <v>15100</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n"/>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>绍兴袍江经济技术开发区投资发展集团有限公司</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E48" s="4" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>徐志庆</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市未来公用事业产业发展有限公司</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E49" s="9" t="n">
+        <v>116000</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>傅强</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市未来公用事业产业发展有限公司</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="n">
+        <v>28000</v>
+      </c>
+      <c r="E50" s="9" t="n">
+        <v>166000</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>徐志庆</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>中国农业银行股份有限公司绍兴分行</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E51" s="9" t="n">
+        <v>116000</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>徐琦</t>
+        </is>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>中国农业银行股份有限公司绍兴分行</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E52" s="9" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>傅强</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>新安县国宸置业有限公司</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E53" s="9" t="n">
+        <v>166000</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>朱云</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>绍兴中洲园林建设有限公司</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="n">
+        <v>40000</v>
+      </c>
+      <c r="E54" s="9" t="n">
+        <v>105522.4</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="n"/>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>薛银辉（个人）</t>
+        </is>
+      </c>
+      <c r="D55" s="9" t="n">
+        <v>40000</v>
+      </c>
+      <c r="E55" s="4" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>傅强</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>陈国柱，丁朝阳，赵月安，刘锦根</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E56" s="9" t="n">
+        <v>166000</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>徐志庆</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市登灏建筑装饰工程有限公司</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="n">
+        <v>19000</v>
+      </c>
+      <c r="E57" s="9" t="n">
+        <v>116000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>孙奕</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市登灏建筑装饰工程有限公司</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="n">
+        <v>18000</v>
+      </c>
+      <c r="E58" s="9" t="n">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="n"/>
+      <c r="C59" s="4" t="n"/>
+      <c r="D59" s="6" t="n">
+        <v>924822.4</v>
+      </c>
+      <c r="E59" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1101,7 +2357,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2025年度开具发票截止2025年12月律师未收款明细表</t>
+          <t>2024年度开具发票截止2024年12月律师未收款明细表</t>
         </is>
       </c>
     </row>
@@ -1144,6 +2400,315 @@
         <v>0</v>
       </c>
       <c r="E4" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>浙江震天律师事务所</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2023年度开具发票截止2023年12月律师未收款明细表</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>姓名</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>发票开具月份</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>对方抬头</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>未收款金额</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>周士杰</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>6月</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>浙江东厦建工集团有限公司</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>韩丽敏</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>6月</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>浙江东厦建工集团有限公司</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E6" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>浙江震天律师事务所</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2022年度开具发票截止2022年12月律师未收款明细表</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>姓名</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>发票开具月份</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>对方抬头</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>未收款金额</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>浙江震天律师事务所</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2020年度开具发票截止2020年12月律师未收款明细表</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>姓名</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>发票开具月份</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>对方抬头</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>未收款金额</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>丁飚</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>绍兴市越城区房地产管理处</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>25000</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="6" t="n">
+        <v>25000</v>
+      </c>
+      <c r="E5" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>